<commit_message>
Trim to 40 deals under $11M, sort by cap, add OM PDFs and photos
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/files/30-3750-midvale-ave.xlsx
+++ b/files/30-3750-midvale-ave.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iniculete\LAAA-Deploys\onmarket\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D7EEA59C-E82D-4D10-8844-B6439DBB27B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E47558AD-4D28-419C-8D65-4274F0E7B4FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{443B15CE-C1E9-4BD7-9B7A-A03C826C37FE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{FA2CD07C-EDB5-44E0-9CDC-3D54D779B5D4}"/>
   </bookViews>
   <sheets>
     <sheet name="Assumptions" sheetId="1" r:id="rId1"/>
     <sheet name="30 3750 Midvale Ave" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'30 3750 Midvale Ave'!$A$1:$N$80</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'30 3750 Midvale Ave'!$A$1:$N$78</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -648,7 +648,7 @@
         <xdr:cNvPr id="2" name="Image 1" descr="Picture">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8686E4D4-A6CB-4D2E-A4C4-C10A06CA093C}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7F535EFC-F1D0-437D-B7DA-81E838D080CB}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -959,7 +959,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1A4C523-F5E3-4C41-BD8B-4147B1AE089A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{539B0014-690A-4AC1-AF5B-F42499376926}">
   <dimension ref="A1:C40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1328,7 +1328,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F56AC93B-4AD3-49D0-9449-C77982E65253}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37913C30-F395-4D88-976A-5C9D6C51A2B0}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -2141,11 +2141,11 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A3" r:id="rId1" xr:uid="{9A5DCA15-A720-4F62-949E-5096A55247F0}"/>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{6782196B-E58B-458F-AE70-8BF07FB7571C}"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.27777777777777779" right="0.27777777777777779" top="0.34722222222222221" bottom="0.34722222222222221" header="0.5" footer="0.5"/>
-  <pageSetup scale="59" fitToHeight="2" orientation="landscape" r:id="rId2"/>
+  <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.5" footer="0.5"/>
+  <pageSetup scale="50" orientation="landscape" r:id="rId2"/>
   <drawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>